<commit_message>
Update imports data auto update selling
</commit_message>
<xml_diff>
--- a/sqms_apps/static/format-upload/template-format-hos-before-import.xlsx
+++ b/sqms_apps/static/format-upload/template-format-hos-before-import.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meinardus.bria\django_project\alpha\sqms_apps\static\format-upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7E035A-6016-4D9B-8E31-D1C682FBF67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CB2C71-9EA2-4707-9094-DE8096800B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="524" xr2:uid="{164D2D34-7551-47B0-9F6A-8815E64D8F5F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="524" xr2:uid="{164D2D34-7551-47B0-9F6A-8815E64D8F5F}"/>
   </bookViews>
   <sheets>
     <sheet name="Format HOS" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Format HOS'!$A$1:$S$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Format HOS'!$A$1:$R$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,6 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Meinardus Bria</author>
-    <author>tc={FE09BA62-4126-4532-BB25-F2E4B4B4EF97}</author>
   </authors>
   <commentList>
     <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{501997AB-239F-41FD-8DED-5EA24661CEDE}">
@@ -69,15 +68,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="1" shapeId="0" xr:uid="{FE09BA62-4126-4532-BB25-F2E4B4B4EF97}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    harus : LIM</t>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{603E0113-CE79-4745-A6A0-7E46B24E0D6B}">
+    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{603E0113-CE79-4745-A6A0-7E46B24E0D6B}">
       <text>
         <r>
           <rPr>
@@ -112,7 +103,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0" xr:uid="{CFA1758A-60B9-4440-BB6F-6D9203EA36E5}">
+    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{CFA1758A-60B9-4440-BB6F-6D9203EA36E5}">
       <text>
         <r>
           <rPr>
@@ -152,7 +143,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>shift</t>
   </si>
@@ -224,9 +215,6 @@
   </si>
   <si>
     <t>FPP_HY</t>
-  </si>
-  <si>
-    <t>adjust_sale</t>
   </si>
   <si>
     <t>SL_01</t>
@@ -444,7 +432,7 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="5"/>
@@ -525,7 +513,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="4" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="60% - Accent2" xfId="8" builtinId="36"/>
@@ -553,9 +540,7 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Meinardus Bria" id="{394ADDEE-1CAA-4275-AD26-E1E56599289F}" userId="Meinardus Bria" providerId="None"/>
-</personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -853,17 +838,9 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="S1" dT="2024-05-30T01:14:32.08" personId="{394ADDEE-1CAA-4275-AD26-E1E56599289F}" id="{FE09BA62-4126-4532-BB25-F2E4B4B4EF97}">
-    <text>harus : LIM</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{675D438A-BC23-488B-AFE3-E8314FA5CCB8}">
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -884,15 +861,14 @@
     <col min="16" max="16" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11" style="7" customWidth="1"/>
     <col min="18" max="18" width="11.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.140625" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.140625" customWidth="1"/>
-    <col min="24" max="25" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" customWidth="1"/>
+    <col min="23" max="24" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>2</v>
       </c>
@@ -947,24 +923,21 @@
       <c r="R1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="8" t="s">
-        <v>24</v>
-      </c>
+      <c r="S1" s="2"/>
       <c r="T1" s="2"/>
       <c r="U1" s="2"/>
       <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="12" t="s">
+      <c r="W1" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="Y1" s="12"/>
+      <c r="X1" s="12"/>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C2" s="28" t="s">
         <v>4</v>
@@ -991,17 +964,17 @@
         <v>45658</v>
       </c>
       <c r="K2" s="28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L2" s="28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M2" s="28" t="s">
         <v>23</v>
       </c>
       <c r="N2" s="31"/>
       <c r="O2" s="31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P2" s="32" t="s">
         <v>12</v>
@@ -1010,37 +983,34 @@
         <v>22</v>
       </c>
       <c r="R2" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="S2" s="34" t="s">
-        <v>4</v>
+        <v>24</v>
+      </c>
+      <c r="S2" s="1" t="str">
+        <f>TEXT(G2, "yyyy-mm-dd")</f>
+        <v>2025-01-01</v>
       </c>
       <c r="T2" s="1" t="str">
-        <f t="shared" ref="T2:T4" si="0">TEXT(G2, "yyyy-mm-dd")</f>
+        <f>TEXT(G2, "hh:mm:ss")</f>
+        <v>05:54:32</v>
+      </c>
+      <c r="U2" s="3" t="str">
+        <f>TEXT(H2, "yyyy-mm-dd")</f>
         <v>2025-01-01</v>
       </c>
-      <c r="U2" s="1" t="str">
-        <f t="shared" ref="U2:U4" si="1">TEXT(G2, "hh:mm:ss")</f>
-        <v>05:54:32</v>
-      </c>
       <c r="V2" s="3" t="str">
-        <f t="shared" ref="V2:V4" si="2">TEXT(H2, "yyyy-mm-dd")</f>
-        <v>2025-01-01</v>
-      </c>
-      <c r="W2" s="3" t="str">
-        <f t="shared" ref="W2:W4" si="3">TEXT(H2, "hh:mm:ss")</f>
+        <f>TEXT(H2, "hh:mm:ss")</f>
         <v>06:05:38</v>
       </c>
+      <c r="W2" s="15">
+        <f t="shared" ref="W2:W4" si="0">DATEVALUE(S2)+TIMEVALUE(T2)</f>
+        <v>45658.246203703704</v>
+      </c>
       <c r="X2" s="15">
-        <f t="shared" ref="X2:X4" si="4">DATEVALUE(T2)+TIMEVALUE(U2)</f>
-        <v>45658.246203703704</v>
-      </c>
-      <c r="Y2" s="15">
-        <f t="shared" ref="Y2:Y4" si="5">DATEVALUE(V2)+TIMEVALUE(W2)</f>
+        <f t="shared" ref="X2:X4" si="1">DATEVALUE(U2)+TIMEVALUE(V2)</f>
         <v>45658.253912037035</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="26"/>
       <c r="B3" s="27"/>
       <c r="C3" s="28"/>
@@ -1059,33 +1029,32 @@
       <c r="P3" s="32"/>
       <c r="Q3" s="28"/>
       <c r="R3" s="33"/>
-      <c r="S3" s="34"/>
+      <c r="S3" s="1" t="str">
+        <f>TEXT(G3, "yyyy-mm-dd")</f>
+        <v>1900-01-00</v>
+      </c>
       <c r="T3" s="1" t="str">
+        <f>TEXT(G3, "hh:mm:ss")</f>
+        <v>00:00:00</v>
+      </c>
+      <c r="U3" s="3" t="str">
+        <f>TEXT(H3, "yyyy-mm-dd")</f>
+        <v>1900-01-00</v>
+      </c>
+      <c r="V3" s="3" t="str">
+        <f>TEXT(H3, "hh:mm:ss")</f>
+        <v>00:00:00</v>
+      </c>
+      <c r="W3" s="15" t="e">
         <f t="shared" si="0"/>
-        <v>1900-01-00</v>
-      </c>
-      <c r="U3" s="1" t="str">
+        <v>#VALUE!</v>
+      </c>
+      <c r="X3" s="15" t="e">
         <f t="shared" si="1"/>
-        <v>00:00:00</v>
-      </c>
-      <c r="V3" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>1900-01-00</v>
-      </c>
-      <c r="W3" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>00:00:00</v>
-      </c>
-      <c r="X3" s="15" t="e">
-        <f t="shared" si="4"/>
         <v>#VALUE!</v>
       </c>
-      <c r="Y3" s="15" t="e">
-        <f t="shared" si="5"/>
-        <v>#VALUE!</v>
-      </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="26"/>
       <c r="B4" s="27"/>
       <c r="C4" s="28"/>
@@ -1104,34 +1073,33 @@
       <c r="P4" s="32"/>
       <c r="Q4" s="28"/>
       <c r="R4" s="33"/>
-      <c r="S4" s="34"/>
+      <c r="S4" s="1" t="str">
+        <f>TEXT(G4, "yyyy-mm-dd")</f>
+        <v>1900-01-00</v>
+      </c>
       <c r="T4" s="1" t="str">
+        <f>TEXT(G4, "hh:mm:ss")</f>
+        <v>00:00:00</v>
+      </c>
+      <c r="U4" s="3" t="str">
+        <f>TEXT(H4, "yyyy-mm-dd")</f>
+        <v>1900-01-00</v>
+      </c>
+      <c r="V4" s="3" t="str">
+        <f>TEXT(H4, "hh:mm:ss")</f>
+        <v>00:00:00</v>
+      </c>
+      <c r="W4" s="15" t="e">
         <f t="shared" si="0"/>
-        <v>1900-01-00</v>
-      </c>
-      <c r="U4" s="1" t="str">
+        <v>#VALUE!</v>
+      </c>
+      <c r="X4" s="15" t="e">
         <f t="shared" si="1"/>
-        <v>00:00:00</v>
-      </c>
-      <c r="V4" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>1900-01-00</v>
-      </c>
-      <c r="W4" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>00:00:00</v>
-      </c>
-      <c r="X4" s="15" t="e">
-        <f t="shared" si="4"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Y4" s="15" t="e">
-        <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S4" xr:uid="{675D438A-BC23-488B-AFE3-E8314FA5CCB8}"/>
+  <autoFilter ref="A1:R4" xr:uid="{675D438A-BC23-488B-AFE3-E8314FA5CCB8}"/>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>

</xml_diff>